<commit_message>
[MODULE_FE, MODULE_BE] feat/fix: fix camera image upload, dynamic canvas and heatmap date filters
</commit_message>
<xml_diff>
--- a/POS_Mau_Test.xlsx
+++ b/POS_Mau_Test.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -440,7 +440,7 @@
         <v>HD0001</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-10T08:15:00Z</v>
+        <v>2026-05-11T01:15:00Z</v>
       </c>
       <c r="C2">
         <v>150000</v>
@@ -466,7 +466,7 @@
         <v>HD0001</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-10T08:15:00Z</v>
+        <v>2026-05-11T01:15:00Z</v>
       </c>
       <c r="C3">
         <v>150000</v>
@@ -492,7 +492,7 @@
         <v>HD0002</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-10T09:30:00Z</v>
+        <v>2026-05-11T02:30:00Z</v>
       </c>
       <c r="C4">
         <v>55000</v>
@@ -518,7 +518,7 @@
         <v>HD0003</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-10T12:05:00Z</v>
+        <v>2026-05-11T05:05:00Z</v>
       </c>
       <c r="C5">
         <v>210000</v>
@@ -539,9 +539,61 @@
         <v>Thẻ tín dụng</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>HD0004</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-05-11T07:20:00Z</v>
+      </c>
+      <c r="C6">
+        <v>320000</v>
+      </c>
+      <c r="D6">
+        <v>20000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Nước ép trái cây</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>45000</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Chuyển khoản</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>HD0005</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-05-11T09:00:00Z</v>
+      </c>
+      <c r="C7">
+        <v>85000</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Bánh tiramisu</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>85000</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Tiền mặt</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>